<commit_message>
feat: build regional gold star schema and reporting layer
</commit_message>
<xml_diff>
--- a/data/raw/singapore/vendor_master.xlsx
+++ b/data/raw/singapore/vendor_master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,11 +439,6 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>vendor_country</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
           <t>active_flag</t>
         </is>
       </c>
@@ -451,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SG-S0001</t>
+          <t>SG-SUP-001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Jarvis and Sons</t>
+          <t>Synthetic Supplier SG 001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Travel Service</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -470,11 +465,6 @@
         </is>
       </c>
       <c r="E2" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -483,30 +473,25 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SG-S0002</t>
+          <t>SG-SUP-002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Perry PLC</t>
+          <t>Synthetic Supplier SG 002</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Ground</t>
+          <t>Airline</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -515,17 +500,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SG-S0003</t>
+          <t>SG-SUP-003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Pham-Gregory</t>
+          <t>Synthetic Supplier SG 003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Airline</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -534,11 +519,6 @@
         </is>
       </c>
       <c r="E4" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -547,30 +527,25 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SG-S0004</t>
+          <t>SG-SUP-004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Carr LLC</t>
+          <t>Synthetic Supplier SG 004</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Travel Service</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -579,17 +554,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SG-S0005</t>
+          <t>SG-SUP-005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Johnson, Cohen and Roberson</t>
+          <t>Synthetic Supplier SG 005</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Hotel</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -598,11 +573,6 @@
         </is>
       </c>
       <c r="E6" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -611,17 +581,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SG-S0006</t>
+          <t>SG-SUP-006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Webb Group</t>
+          <t>Synthetic Supplier SG 006</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Ground Transport</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -631,42 +601,32 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Active</t>
+          <t>Inactive</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SG-S0007</t>
+          <t>SG-SUP-007</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Clay Group</t>
+          <t>Synthetic Supplier SG 007</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Ground Transport</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -675,17 +635,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SG-S0008</t>
+          <t>SG-SUP-008</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Brown Ltd</t>
+          <t>Synthetic Supplier SG 008</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Ground</t>
+          <t>Hotel</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -694,11 +654,6 @@
         </is>
       </c>
       <c r="E9" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -707,30 +662,25 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SG-S0009</t>
+          <t>SG-SUP-009</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Smith-Oneill</t>
+          <t>Synthetic Supplier SG 009</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Hotel</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -739,30 +689,25 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SG-S0010</t>
+          <t>SG-SUP-010</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Saunders, Ray and Cunningham</t>
+          <t>Synthetic Supplier SG 010</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Airline</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -771,30 +716,25 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SG-S0011</t>
+          <t>SG-SUP-011</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Marks, Stone and Watts</t>
+          <t>Synthetic Supplier SG 011</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Ground</t>
+          <t>Hotel</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -803,12 +743,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SG-S0012</t>
+          <t>SG-SUP-012</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Davis, Stanley and Wright</t>
+          <t>Synthetic Supplier SG 012</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -822,11 +762,6 @@
         </is>
       </c>
       <c r="E13" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -835,30 +770,25 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SG-S0013</t>
+          <t>SG-SUP-013</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Alvarado-Davidson</t>
+          <t>Synthetic Supplier SG 013</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Ground Transport</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -867,17 +797,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SG-S0014</t>
+          <t>SG-SUP-014</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Combs PLC</t>
+          <t>Synthetic Supplier SG 014</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Ground Transport</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -886,11 +816,6 @@
         </is>
       </c>
       <c r="E15" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -899,12 +824,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SG-S0015</t>
+          <t>SG-SUP-015</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Brown, Schneider and Moore</t>
+          <t>Synthetic Supplier SG 015</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -914,15 +839,10 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -931,30 +851,25 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SG-S0016</t>
+          <t>SG-SUP-016</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Christian-Booth</t>
+          <t>Synthetic Supplier SG 016</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Travel Service</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -963,17 +878,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SG-S0017</t>
+          <t>SG-SUP-017</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Walton LLC</t>
+          <t>Synthetic Supplier SG 017</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Travel Service</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -982,11 +897,6 @@
         </is>
       </c>
       <c r="E18" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -995,30 +905,25 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SG-S0018</t>
+          <t>SG-SUP-018</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Rivera LLC</t>
+          <t>Synthetic Supplier SG 018</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Airline</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1027,17 +932,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SG-S0019</t>
+          <t>SG-SUP-019</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Hunter PLC</t>
+          <t>Synthetic Supplier SG 019</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Hotel</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1046,11 +951,6 @@
         </is>
       </c>
       <c r="E20" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1059,12 +959,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SG-S0020</t>
+          <t>SG-SUP-020</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Gray, Montoya and Miller</t>
+          <t>Synthetic Supplier SG 020</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1074,15 +974,10 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1091,30 +986,25 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SG-S0021</t>
+          <t>SG-SUP-021</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Solis-West</t>
+          <t>Synthetic Supplier SG 021</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Ground</t>
+          <t>Hotel</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1123,30 +1013,25 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SG-S0022</t>
+          <t>SG-SUP-022</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>West-Wilson</t>
+          <t>Synthetic Supplier SG 022</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Hotel</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1155,30 +1040,25 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SG-S0023</t>
+          <t>SG-SUP-023</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mcgee-Smith</t>
+          <t>Synthetic Supplier SG 023</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Airline</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1187,12 +1067,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SG-S0024</t>
+          <t>SG-SUP-024</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Gutierrez-Hawkins</t>
+          <t>Synthetic Supplier SG 024</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1202,15 +1082,10 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1219,17 +1094,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SG-S0025</t>
+          <t>SG-SUP-025</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Petersen PLC</t>
+          <t>Synthetic Supplier SG 025</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Ground Transport</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1238,11 +1113,6 @@
         </is>
       </c>
       <c r="E26" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1251,12 +1121,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SG-S0026</t>
+          <t>SG-SUP-026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Walsh, Wu and Hart</t>
+          <t>Synthetic Supplier SG 026</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1270,11 +1140,6 @@
         </is>
       </c>
       <c r="E27" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1283,17 +1148,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SG-S0027</t>
+          <t>SG-SUP-027</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Powers, Clements and Cox</t>
+          <t>Synthetic Supplier SG 027</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Ground</t>
+          <t>Ground Transport</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1302,11 +1167,6 @@
         </is>
       </c>
       <c r="E28" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1315,17 +1175,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SG-S0028</t>
+          <t>SG-SUP-028</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Velasquez Group</t>
+          <t>Synthetic Supplier SG 028</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Travel Service</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1334,11 +1194,6 @@
         </is>
       </c>
       <c r="E29" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1347,17 +1202,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SG-S0029</t>
+          <t>SG-SUP-029</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Castro-Harvey</t>
+          <t>Synthetic Supplier SG 029</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Travel Service</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1366,11 +1221,6 @@
         </is>
       </c>
       <c r="E30" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1379,30 +1229,25 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SG-S0030</t>
+          <t>SG-SUP-030</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Moran-Cox</t>
+          <t>Synthetic Supplier SG 030</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Ground Transport</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1411,17 +1256,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SG-S0031</t>
+          <t>SG-SUP-031</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Wilson-Malone</t>
+          <t>Synthetic Supplier SG 031</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Travel Service</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1430,11 +1275,6 @@
         </is>
       </c>
       <c r="E32" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1443,17 +1283,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SG-S0032</t>
+          <t>SG-SUP-032</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Smith LLC</t>
+          <t>Synthetic Supplier SG 032</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Travel Service</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1462,11 +1302,6 @@
         </is>
       </c>
       <c r="E33" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1475,17 +1310,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SG-S0033</t>
+          <t>SG-SUP-033</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Brandt, Carter and Boyd</t>
+          <t>Synthetic Supplier SG 033</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Hotel</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1494,11 +1329,6 @@
         </is>
       </c>
       <c r="E34" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1507,30 +1337,25 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SG-S0034</t>
+          <t>SG-SUP-034</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Rodriguez, Prince and Vasquez</t>
+          <t>Synthetic Supplier SG 034</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Airline</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1539,17 +1364,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SG-S0035</t>
+          <t>SG-SUP-035</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Newton, Ortiz and King</t>
+          <t>Synthetic Supplier SG 035</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Travel Service</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1558,11 +1383,6 @@
         </is>
       </c>
       <c r="E36" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1571,17 +1391,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SG-S0036</t>
+          <t>SG-SUP-036</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Lopez Group</t>
+          <t>Synthetic Supplier SG 036</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Ground</t>
+          <t>Airline</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1590,11 +1410,6 @@
         </is>
       </c>
       <c r="E37" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1603,30 +1418,25 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SG-S0037</t>
+          <t>SG-SUP-037</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Bryant and Sons</t>
+          <t>Synthetic Supplier SG 037</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Hotel</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1635,30 +1445,25 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SG-S0038</t>
+          <t>SG-SUP-038</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Morgan, Sherman and Williams</t>
+          <t>Synthetic Supplier SG 038</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Airline</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1667,17 +1472,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SG-S0039</t>
+          <t>SG-SUP-039</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Monroe, Chapman and Barton</t>
+          <t>Synthetic Supplier SG 039</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Hotel</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1686,11 +1491,6 @@
         </is>
       </c>
       <c r="E40" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1699,17 +1499,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SG-S0040</t>
+          <t>SG-SUP-040</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Ellis-Lawrence</t>
+          <t>Synthetic Supplier SG 040</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Ground Transport</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1718,11 +1518,6 @@
         </is>
       </c>
       <c r="E41" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1731,17 +1526,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SG-S0041</t>
+          <t>SG-SUP-041</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Taylor, Porter and Moreno</t>
+          <t>Synthetic Supplier SG 041</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Airline</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1750,11 +1545,6 @@
         </is>
       </c>
       <c r="E42" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1763,17 +1553,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SG-S0042</t>
+          <t>SG-SUP-042</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Tran Group</t>
+          <t>Synthetic Supplier SG 042</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Ground</t>
+          <t>Travel Service</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1782,11 +1572,6 @@
         </is>
       </c>
       <c r="E43" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1795,30 +1580,25 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SG-S0043</t>
+          <t>SG-SUP-043</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Webb, Romero and Morse</t>
+          <t>Synthetic Supplier SG 043</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Travel Service</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1827,17 +1607,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SG-S0044</t>
+          <t>SG-SUP-044</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Holt and Sons</t>
+          <t>Synthetic Supplier SG 044</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Hotel</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1846,11 +1626,6 @@
         </is>
       </c>
       <c r="E45" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1859,30 +1634,25 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SG-S0045</t>
+          <t>SG-SUP-045</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Ochoa, Garcia and Sandoval</t>
+          <t>Synthetic Supplier SG 045</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Travel Service</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1891,30 +1661,25 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>SG-S0046</t>
+          <t>SG-SUP-046</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Andrade, Gordon and Cruz</t>
+          <t>Synthetic Supplier SG 046</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Ground Transport</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1923,30 +1688,25 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SG-S0047</t>
+          <t>SG-SUP-047</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Moon, Farmer and Hill</t>
+          <t>Synthetic Supplier SG 047</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Travel Service</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1955,17 +1715,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SG-S0048</t>
+          <t>SG-SUP-048</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Waller-Chavez</t>
+          <t>Synthetic Supplier SG 048</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Airline</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1974,11 +1734,6 @@
         </is>
       </c>
       <c r="E49" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -1987,17 +1742,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SG-S0049</t>
+          <t>SG-SUP-049</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Taylor PLC</t>
+          <t>Synthetic Supplier SG 049</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Ground Transport</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2006,11 +1761,6 @@
         </is>
       </c>
       <c r="E50" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -2019,30 +1769,25 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SG-S0050</t>
+          <t>SG-SUP-050</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Tanner, Hunt and Cameron</t>
+          <t>Synthetic Supplier SG 050</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Ground</t>
+          <t>Airline</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -2051,17 +1796,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SG-S0051</t>
+          <t>SG-SUP-051</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Valencia, Joseph and Walls</t>
+          <t>Synthetic Supplier SG 051</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Airline</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2070,11 +1815,6 @@
         </is>
       </c>
       <c r="E52" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -2083,62 +1823,52 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SG-S0052</t>
+          <t>SG-SUP-052</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Robinson, Clark and Klein</t>
+          <t>Synthetic Supplier SG 052</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Hotel</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>Active</t>
+          <t>Inactive</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SG-S0053</t>
+          <t>SG-SUP-053</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Reed, Chambers and Zavala</t>
+          <t>Synthetic Supplier SG 053</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Ground Transport</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -2147,17 +1877,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SG-S0054</t>
+          <t>SG-SUP-054</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Hester, Thompson and Daniels</t>
+          <t>Synthetic Supplier SG 054</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Ground Transport</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2167,29 +1897,24 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>Active</t>
+          <t>Inactive</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SG-S0055</t>
+          <t>SG-SUP-055</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Morris, Wilson and Bell</t>
+          <t>Synthetic Supplier SG 055</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Ground Transport</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2198,11 +1923,6 @@
         </is>
       </c>
       <c r="E56" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -2211,17 +1931,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>SG-S0056</t>
+          <t>SG-SUP-056</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Aguilar-Bender</t>
+          <t>Synthetic Supplier SG 056</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Ground</t>
+          <t>Hotel</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2230,11 +1950,6 @@
         </is>
       </c>
       <c r="E57" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -2243,30 +1958,25 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>SG-S0057</t>
+          <t>SG-SUP-057</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Butler, Adkins and Skinner</t>
+          <t>Synthetic Supplier SG 057</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Ground Transport</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -2275,17 +1985,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>SG-S0058</t>
+          <t>SG-SUP-058</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Rich-Henderson</t>
+          <t>Synthetic Supplier SG 058</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Air</t>
+          <t>Ground Transport</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2294,11 +2004,6 @@
         </is>
       </c>
       <c r="E59" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -2307,17 +2012,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>SG-S0059</t>
+          <t>SG-SUP-059</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Mills Inc</t>
+          <t>Synthetic Supplier SG 059</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Ground</t>
+          <t>Airline</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2326,11 +2031,6 @@
         </is>
       </c>
       <c r="E60" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -2339,17 +2039,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>SG-S0060</t>
+          <t>SG-SUP-060</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Thomas-Santiago</t>
+          <t>Synthetic Supplier SG 060</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Travel Service</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2358,11 +2058,6 @@
         </is>
       </c>
       <c r="E61" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
         <is>
           <t>Active</t>
         </is>

</xml_diff>